<commit_message>
Vérités : alerte PE012 écrite comme au journal, alertes attendues de PE011
- 223111PE012 Alertes_attendues E2 : texte exact du journal, sans la consigne autour
- 223111PE011 : feuille Alertes_attendues (TYPE absent p. 104, contrôle INDICE impossible)
- 6A23111PE133 RC 20 inchangé (« TRANS » sans point, prouvé par Verite_positions)
- Journal : résultats du passage réel du 2026-10-05

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/223111PE011_extrait_verite.xlsx
+++ b/tests/fixtures/223111PE011_extrait_verite.xlsx
@@ -9,7 +9,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISEZ-MOI" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verite_tableaux" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verite_pieds" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verite_positions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alertes_attendues" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verite_positions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +43,13 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +66,11 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -73,11 +84,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7376,6 +7391,122 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Page extrait</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Page document</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Ligne</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Colonne</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Alerte attendue</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Pourquoi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>pied</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>TYPE</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>champ TYPE absent du pied, laissé vide : page(s) 104</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Le pied de la page 104 (CABLE : RESERVE) n'imprime pas de TYPE : rien n'est inventé</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>1 à 10</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>1 à 123</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>garde</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>INDICE</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>contrôle INDICE impossible : aucune liste de révisions lue sur une page de garde</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>L'extrait n'a pas de page de garde : aucune liste de révisions pour contrôler les INDICE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>